<commit_message>
Fix truncated CSV header bug in features/extract.py and add HPSS replication study
The per-segment features CSV wrote its header once, based on whichever
song finished first under Pool.imap_unordered; songs with more segments
than that one produced rows wider than the header, breaking pd.read_csv.
run_parallel() now buffers all per-song frames and writes the CSV once
with a header that's the real union of every seg_N column. Also fixes a
related bug where an existing-but-empty summary CSV was treated as
already having a header.

Add research/hpss_replication_96/: re-runs the HPSS/perc_ratio removal
analysis from the root README against the current real 96-song dataset
(kernel-size validation, feature importance, ablation test, worker
benchmarks with and without HPSS), with raw evidence CSVs per phase.
</commit_message>
<xml_diff>
--- a/data/audio/_canciones_rock_english.xlsx
+++ b/data/audio/_canciones_rock_english.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\JOli\Documents\Projects\datalab-music-mood\music-tagger-benchmark\data\audio\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3D5658E3-8D67-4D2F-B07B-2BEB3BB0D24A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5EE942B1-CF00-4DF1-804B-876B84D14A4E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="9990" yWindow="5910" windowWidth="21630" windowHeight="8610" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Dinamica" sheetId="3" r:id="rId1"/>
@@ -19,7 +19,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'AI-evaluation'!$A$1:$B$299</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">data!$A$1:$E$419</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">data!$A$1:$D$426</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <pivotCaches>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2286" uniqueCount="611">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2313" uniqueCount="617">
   <si>
     <t>10cc - I'm Not In Love</t>
   </si>
@@ -1874,7 +1874,25 @@
     <t>Count of categorico</t>
   </si>
   <si>
-    <t>procesar</t>
+    <t>Metallica - Battery (Remastered)</t>
+  </si>
+  <si>
+    <t>Metallica - Damage, Inc. (Remastered)</t>
+  </si>
+  <si>
+    <t>Metallica - Leper Messiah (Remastered)</t>
+  </si>
+  <si>
+    <t>Metallica - Master of Puppets (Remastered)</t>
+  </si>
+  <si>
+    <t>Metallica - Orion (Remastered)</t>
+  </si>
+  <si>
+    <t>Metallica - The Thing That Should Not Be (Remastered)</t>
+  </si>
+  <si>
+    <t>Metallica - Welcome Home (Sanitarium) (Remastered)</t>
   </si>
 </sst>
 </file>
@@ -1952,7 +1970,7 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="JOli" refreshedDate="46238.599384837966" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="418" xr:uid="{1ECF6FD6-748B-4665-B4C9-9C2AFF903A4D}">
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="JOli" refreshedDate="46245.872911342594" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="418" xr:uid="{1ECF6FD6-748B-4665-B4C9-9C2AFF903A4D}">
   <cacheSource type="worksheet">
     <worksheetSource ref="A1:D419" sheet="data"/>
   </cacheSource>
@@ -2994,7 +3012,7 @@
     <s v="ACDC - Highway to Hell"/>
     <s v="hard_rock"/>
     <x v="2"/>
-    <x v="0"/>
+    <x v="3"/>
   </r>
   <r>
     <s v="Boney M. - Gotta Go Home"/>
@@ -3006,19 +3024,19 @@
     <s v="Scorpions - Still Loving You"/>
     <s v="hard_rock"/>
     <x v="2"/>
-    <x v="0"/>
+    <x v="4"/>
   </r>
   <r>
     <s v="ACDC - Thunderstruck"/>
     <s v="hard_rock"/>
     <x v="2"/>
-    <x v="0"/>
+    <x v="3"/>
   </r>
   <r>
     <s v="Aerosmith - Dream On"/>
     <s v="hard_rock"/>
     <x v="2"/>
-    <x v="0"/>
+    <x v="4"/>
   </r>
   <r>
     <s v="Michael Jackson - Beat It"/>
@@ -3034,7 +3052,7 @@
   </r>
   <r>
     <s v="Molchat Doma - Судно (Борис Рыжий)"/>
-    <s v="hard-rock"/>
+    <s v="hard_rock"/>
     <x v="2"/>
     <x v="0"/>
   </r>
@@ -3052,9 +3070,9 @@
   </r>
   <r>
     <s v="Aerosmith - Cryin'"/>
-    <s v="hard-rock"/>
-    <x v="2"/>
-    <x v="0"/>
+    <s v="hard_rock"/>
+    <x v="2"/>
+    <x v="3"/>
   </r>
   <r>
     <s v="Ozzy Osbourne - No More Tears"/>
@@ -4894,7 +4912,7 @@
         <v>602</v>
       </c>
       <c r="B4">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
@@ -4926,7 +4944,7 @@
         <v>603</v>
       </c>
       <c r="B8">
-        <v>21</v>
+        <v>23</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
@@ -4934,7 +4952,7 @@
         <v>606</v>
       </c>
       <c r="B9">
-        <v>157</v>
+        <v>152</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
@@ -4952,7 +4970,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:N419"/>
+  <dimension ref="A1:D426"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="97.28515625" bestFit="1" customWidth="1"/>
@@ -4961,7 +4979,7 @@
     <col min="4" max="4" width="25.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>418</v>
       </c>
@@ -4974,11 +4992,8 @@
       <c r="D1" t="s">
         <v>605</v>
       </c>
-      <c r="E1" t="s">
-        <v>610</v>
-      </c>
-    </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>144</v>
       </c>
@@ -4992,7 +5007,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>147</v>
       </c>
@@ -5006,7 +5021,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>145</v>
       </c>
@@ -5019,14 +5034,8 @@
       <c r="D4" t="s">
         <v>606</v>
       </c>
-      <c r="E4" t="b">
-        <v>1</v>
-      </c>
-      <c r="M4">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>143</v>
       </c>
@@ -5040,7 +5049,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>415</v>
       </c>
@@ -5054,7 +5063,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>360</v>
       </c>
@@ -5067,18 +5076,8 @@
       <c r="D7" t="s">
         <v>606</v>
       </c>
-      <c r="L7">
-        <v>25</v>
-      </c>
-      <c r="M7">
-        <v>7.1999999999999993</v>
-      </c>
-      <c r="N7">
-        <f>+(L7*M7)/60</f>
-        <v>2.9999999999999996</v>
-      </c>
-    </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>316</v>
       </c>
@@ -5092,7 +5091,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>315</v>
       </c>
@@ -5106,7 +5105,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>235</v>
       </c>
@@ -5120,7 +5119,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>237</v>
       </c>
@@ -5134,7 +5133,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>373</v>
       </c>
@@ -5148,7 +5147,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="13" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>139</v>
       </c>
@@ -5162,7 +5161,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>209</v>
       </c>
@@ -5176,7 +5175,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>1</v>
       </c>
@@ -5190,7 +5189,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>141</v>
       </c>
@@ -5876,7 +5875,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="65" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
         <v>334</v>
       </c>
@@ -5890,7 +5889,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="66" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
         <v>187</v>
       </c>
@@ -5903,11 +5902,8 @@
       <c r="D66" t="s">
         <v>606</v>
       </c>
-      <c r="E66" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="67" spans="1:5" x14ac:dyDescent="0.25">
+    </row>
+    <row r="67" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
         <v>105</v>
       </c>
@@ -5921,7 +5917,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="68" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
         <v>324</v>
       </c>
@@ -5935,7 +5931,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="69" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
         <v>267</v>
       </c>
@@ -5949,7 +5945,7 @@
         <v>602</v>
       </c>
     </row>
-    <row r="70" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
         <v>102</v>
       </c>
@@ -5963,7 +5959,7 @@
         <v>604</v>
       </c>
     </row>
-    <row r="71" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
         <v>119</v>
       </c>
@@ -5977,7 +5973,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="72" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
         <v>269</v>
       </c>
@@ -5991,7 +5987,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="73" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
         <v>208</v>
       </c>
@@ -6005,7 +6001,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="74" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
         <v>158</v>
       </c>
@@ -6019,7 +6015,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="75" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
         <v>181</v>
       </c>
@@ -6033,7 +6029,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="76" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
         <v>241</v>
       </c>
@@ -6047,7 +6043,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="77" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
         <v>306</v>
       </c>
@@ -6061,7 +6057,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="78" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
         <v>178</v>
       </c>
@@ -6075,7 +6071,7 @@
         <v>604</v>
       </c>
     </row>
-    <row r="79" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
         <v>30</v>
       </c>
@@ -6089,7 +6085,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="80" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
         <v>66</v>
       </c>
@@ -6103,7 +6099,7 @@
         <v>604</v>
       </c>
     </row>
-    <row r="81" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
         <v>73</v>
       </c>
@@ -6117,7 +6113,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="82" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
         <v>99</v>
       </c>
@@ -6131,7 +6127,7 @@
         <v>604</v>
       </c>
     </row>
-    <row r="83" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
         <v>100</v>
       </c>
@@ -6145,7 +6141,7 @@
         <v>602</v>
       </c>
     </row>
-    <row r="84" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
         <v>103</v>
       </c>
@@ -6159,7 +6155,7 @@
         <v>600</v>
       </c>
     </row>
-    <row r="85" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
         <v>104</v>
       </c>
@@ -6173,7 +6169,7 @@
         <v>600</v>
       </c>
     </row>
-    <row r="86" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
         <v>137</v>
       </c>
@@ -6184,10 +6180,10 @@
         <v>595</v>
       </c>
       <c r="D86" t="s">
-        <v>606</v>
-      </c>
-    </row>
-    <row r="87" spans="1:5" x14ac:dyDescent="0.25">
+        <v>600</v>
+      </c>
+    </row>
+    <row r="87" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
         <v>136</v>
       </c>
@@ -6198,10 +6194,10 @@
         <v>595</v>
       </c>
       <c r="D87" t="s">
-        <v>606</v>
-      </c>
-    </row>
-    <row r="88" spans="1:5" x14ac:dyDescent="0.25">
+        <v>600</v>
+      </c>
+    </row>
+    <row r="88" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
         <v>173</v>
       </c>
@@ -6215,7 +6211,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="89" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
         <v>174</v>
       </c>
@@ -6229,7 +6225,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="90" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
         <v>3</v>
       </c>
@@ -6243,7 +6239,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="91" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
         <v>6</v>
       </c>
@@ -6257,7 +6253,7 @@
         <v>600</v>
       </c>
     </row>
-    <row r="92" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
         <v>7</v>
       </c>
@@ -6271,7 +6267,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="93" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
         <v>175</v>
       </c>
@@ -6285,7 +6281,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="94" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
         <v>190</v>
       </c>
@@ -6299,7 +6295,7 @@
         <v>600</v>
       </c>
     </row>
-    <row r="95" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
         <v>191</v>
       </c>
@@ -6312,11 +6308,8 @@
       <c r="D95" t="s">
         <v>606</v>
       </c>
-      <c r="E95" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="96" spans="1:5" x14ac:dyDescent="0.25">
+    </row>
+    <row r="96" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
         <v>250</v>
       </c>
@@ -6330,7 +6323,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="97" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
         <v>314</v>
       </c>
@@ -6344,7 +6337,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="98" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
         <v>400</v>
       </c>
@@ -6358,7 +6351,7 @@
         <v>600</v>
       </c>
     </row>
-    <row r="99" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
         <v>410</v>
       </c>
@@ -6372,7 +6365,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="100" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
         <v>42</v>
       </c>
@@ -6386,7 +6379,7 @@
         <v>600</v>
       </c>
     </row>
-    <row r="101" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
         <v>56</v>
       </c>
@@ -6399,11 +6392,8 @@
       <c r="D101" t="s">
         <v>606</v>
       </c>
-      <c r="E101" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="102" spans="1:5" x14ac:dyDescent="0.25">
+    </row>
+    <row r="102" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
         <v>41</v>
       </c>
@@ -6417,7 +6407,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="103" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
         <v>108</v>
       </c>
@@ -6431,7 +6421,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="104" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
         <v>101</v>
       </c>
@@ -6445,7 +6435,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="105" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
         <v>216</v>
       </c>
@@ -6459,7 +6449,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="106" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
         <v>4</v>
       </c>
@@ -6473,7 +6463,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="107" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
         <v>8</v>
       </c>
@@ -6487,7 +6477,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="108" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
         <v>9</v>
       </c>
@@ -6501,7 +6491,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="109" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
         <v>10</v>
       </c>
@@ -6515,7 +6505,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="110" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
         <v>379</v>
       </c>
@@ -6529,7 +6519,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="111" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A111" t="s">
         <v>38</v>
       </c>
@@ -6543,7 +6533,7 @@
         <v>601</v>
       </c>
     </row>
-    <row r="112" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A112" t="s">
         <v>117</v>
       </c>
@@ -6556,11 +6546,8 @@
       <c r="D112" t="s">
         <v>606</v>
       </c>
-      <c r="E112" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="113" spans="1:5" x14ac:dyDescent="0.25">
+    </row>
+    <row r="113" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A113" t="s">
         <v>218</v>
       </c>
@@ -6574,7 +6561,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="114" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A114" t="s">
         <v>253</v>
       </c>
@@ -6588,7 +6575,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="115" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A115" t="s">
         <v>252</v>
       </c>
@@ -6602,7 +6589,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="116" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A116" t="s">
         <v>170</v>
       </c>
@@ -6616,7 +6603,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="117" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A117" t="s">
         <v>310</v>
       </c>
@@ -6630,7 +6617,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="118" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A118" t="s">
         <v>309</v>
       </c>
@@ -6644,7 +6631,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="119" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A119" t="s">
         <v>51</v>
       </c>
@@ -6658,7 +6645,7 @@
         <v>604</v>
       </c>
     </row>
-    <row r="120" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A120" t="s">
         <v>228</v>
       </c>
@@ -6672,7 +6659,7 @@
         <v>602</v>
       </c>
     </row>
-    <row r="121" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A121" t="s">
         <v>179</v>
       </c>
@@ -6686,7 +6673,7 @@
         <v>600</v>
       </c>
     </row>
-    <row r="122" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A122" t="s">
         <v>11</v>
       </c>
@@ -6700,7 +6687,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="123" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A123" t="s">
         <v>221</v>
       </c>
@@ -6714,7 +6701,7 @@
         <v>604</v>
       </c>
     </row>
-    <row r="124" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A124" t="s">
         <v>247</v>
       </c>
@@ -6728,7 +6715,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="125" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A125" t="s">
         <v>246</v>
       </c>
@@ -6742,7 +6729,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="126" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A126" t="s">
         <v>222</v>
       </c>
@@ -6755,11 +6742,8 @@
       <c r="D126" t="s">
         <v>606</v>
       </c>
-      <c r="E126" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="127" spans="1:5" x14ac:dyDescent="0.25">
+    </row>
+    <row r="127" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A127" t="s">
         <v>223</v>
       </c>
@@ -6773,7 +6757,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="128" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A128" t="s">
         <v>189</v>
       </c>
@@ -7235,7 +7219,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="161" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A161" t="s">
         <v>365</v>
       </c>
@@ -7249,7 +7233,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="162" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A162" t="s">
         <v>399</v>
       </c>
@@ -7263,7 +7247,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="163" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A163" t="s">
         <v>115</v>
       </c>
@@ -7277,7 +7261,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="164" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A164" t="s">
         <v>61</v>
       </c>
@@ -7291,7 +7275,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="165" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A165" t="s">
         <v>229</v>
       </c>
@@ -7305,7 +7289,7 @@
         <v>602</v>
       </c>
     </row>
-    <row r="166" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A166" t="s">
         <v>85</v>
       </c>
@@ -7319,7 +7303,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="167" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A167" t="s">
         <v>270</v>
       </c>
@@ -7333,7 +7317,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="168" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A168" t="s">
         <v>12</v>
       </c>
@@ -7344,13 +7328,10 @@
         <v>582</v>
       </c>
       <c r="D168" t="s">
-        <v>606</v>
-      </c>
-      <c r="E168" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="169" spans="1:5" x14ac:dyDescent="0.25">
+        <v>602</v>
+      </c>
+    </row>
+    <row r="169" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A169" t="s">
         <v>63</v>
       </c>
@@ -7364,7 +7345,7 @@
         <v>600</v>
       </c>
     </row>
-    <row r="170" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A170" t="s">
         <v>305</v>
       </c>
@@ -7375,38 +7356,38 @@
         <v>582</v>
       </c>
       <c r="D170" t="s">
-        <v>606</v>
-      </c>
-    </row>
-    <row r="171" spans="1:5" x14ac:dyDescent="0.25">
+        <v>603</v>
+      </c>
+    </row>
+    <row r="171" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A171" t="s">
         <v>13</v>
       </c>
-      <c r="B171" s="3" t="s">
+      <c r="B171" t="s">
         <v>440</v>
       </c>
       <c r="C171" t="s">
         <v>582</v>
       </c>
       <c r="D171" t="s">
-        <v>606</v>
-      </c>
-    </row>
-    <row r="172" spans="1:5" x14ac:dyDescent="0.25">
+        <v>602</v>
+      </c>
+    </row>
+    <row r="172" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A172" t="s">
         <v>20</v>
       </c>
-      <c r="B172" s="3" t="s">
+      <c r="B172" t="s">
         <v>440</v>
       </c>
       <c r="C172" t="s">
         <v>582</v>
       </c>
       <c r="D172" t="s">
-        <v>606</v>
-      </c>
-    </row>
-    <row r="173" spans="1:5" x14ac:dyDescent="0.25">
+        <v>603</v>
+      </c>
+    </row>
+    <row r="173" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A173" t="s">
         <v>214</v>
       </c>
@@ -7420,7 +7401,7 @@
         <v>600</v>
       </c>
     </row>
-    <row r="174" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A174" t="s">
         <v>176</v>
       </c>
@@ -7434,12 +7415,12 @@
         <v>602</v>
       </c>
     </row>
-    <row r="175" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A175" t="s">
         <v>225</v>
       </c>
       <c r="B175" t="s">
-        <v>428</v>
+        <v>440</v>
       </c>
       <c r="C175" t="s">
         <v>582</v>
@@ -7448,7 +7429,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="176" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A176" t="s">
         <v>230</v>
       </c>
@@ -7480,14 +7461,14 @@
       <c r="A178" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="B178" s="3" t="s">
-        <v>428</v>
+      <c r="B178" t="s">
+        <v>440</v>
       </c>
       <c r="C178" t="s">
         <v>582</v>
       </c>
       <c r="D178" t="s">
-        <v>606</v>
+        <v>602</v>
       </c>
     </row>
     <row r="179" spans="1:4" x14ac:dyDescent="0.25">
@@ -7686,7 +7667,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="193" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="193" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A193" t="s">
         <v>196</v>
       </c>
@@ -7700,7 +7681,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="194" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="194" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A194" t="s">
         <v>219</v>
       </c>
@@ -7713,11 +7694,8 @@
       <c r="D194" t="s">
         <v>606</v>
       </c>
-      <c r="E194" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="195" spans="1:5" x14ac:dyDescent="0.25">
+    </row>
+    <row r="195" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A195" t="s">
         <v>220</v>
       </c>
@@ -7731,7 +7709,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="196" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="196" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A196" t="s">
         <v>245</v>
       </c>
@@ -7745,7 +7723,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="197" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="197" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A197" t="s">
         <v>282</v>
       </c>
@@ -7759,7 +7737,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="198" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="198" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A198" t="s">
         <v>283</v>
       </c>
@@ -7773,7 +7751,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="199" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="199" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A199" t="s">
         <v>288</v>
       </c>
@@ -7787,7 +7765,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="200" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="200" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A200" t="s">
         <v>320</v>
       </c>
@@ -7801,7 +7779,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="201" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="201" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A201" t="s">
         <v>376</v>
       </c>
@@ -7815,7 +7793,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="202" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="202" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A202" t="s">
         <v>401</v>
       </c>
@@ -7829,7 +7807,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="203" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="203" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A203" t="s">
         <v>402</v>
       </c>
@@ -7843,7 +7821,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="204" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="204" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A204" t="s">
         <v>406</v>
       </c>
@@ -7857,7 +7835,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="205" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="205" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A205" t="s">
         <v>412</v>
       </c>
@@ -7871,7 +7849,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="206" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="206" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A206" t="s">
         <v>416</v>
       </c>
@@ -7885,7 +7863,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="207" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="207" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A207" t="s">
         <v>363</v>
       </c>
@@ -7899,7 +7877,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="208" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="208" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A208" t="s">
         <v>384</v>
       </c>
@@ -7980,7 +7958,7 @@
         <v>582</v>
       </c>
       <c r="D213" t="s">
-        <v>606</v>
+        <v>601</v>
       </c>
     </row>
     <row r="214" spans="1:4" x14ac:dyDescent="0.25">
@@ -8092,7 +8070,7 @@
         <v>582</v>
       </c>
       <c r="D221" t="s">
-        <v>606</v>
+        <v>601</v>
       </c>
     </row>
     <row r="222" spans="1:4" x14ac:dyDescent="0.25">
@@ -8137,7 +8115,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="225" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="225" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A225" t="s">
         <v>368</v>
       </c>
@@ -8151,7 +8129,7 @@
         <v>604</v>
       </c>
     </row>
-    <row r="226" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="226" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A226" t="s">
         <v>392</v>
       </c>
@@ -8165,7 +8143,7 @@
         <v>604</v>
       </c>
     </row>
-    <row r="227" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="227" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A227" t="s">
         <v>391</v>
       </c>
@@ -8179,7 +8157,7 @@
         <v>604</v>
       </c>
     </row>
-    <row r="228" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="228" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A228" t="s">
         <v>37</v>
       </c>
@@ -8192,11 +8170,8 @@
       <c r="D228" t="s">
         <v>606</v>
       </c>
-      <c r="E228" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="229" spans="1:5" x14ac:dyDescent="0.25">
+    </row>
+    <row r="229" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A229" t="s">
         <v>201</v>
       </c>
@@ -8210,7 +8185,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="230" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="230" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A230" t="s">
         <v>304</v>
       </c>
@@ -8224,7 +8199,7 @@
         <v>604</v>
       </c>
     </row>
-    <row r="231" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="231" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A231" t="s">
         <v>197</v>
       </c>
@@ -8238,7 +8213,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="232" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="232" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A232" t="s">
         <v>124</v>
       </c>
@@ -8252,7 +8227,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="233" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="233" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A233" t="s">
         <v>200</v>
       </c>
@@ -8266,7 +8241,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="234" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="234" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A234" t="s">
         <v>193</v>
       </c>
@@ -8280,7 +8255,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="235" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="235" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A235" t="s">
         <v>29</v>
       </c>
@@ -8294,7 +8269,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="236" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="236" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A236" t="s">
         <v>52</v>
       </c>
@@ -8308,7 +8283,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="237" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="237" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A237" t="s">
         <v>5</v>
       </c>
@@ -8322,7 +8297,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="238" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="238" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A238" t="s">
         <v>21</v>
       </c>
@@ -8336,7 +8311,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="239" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="239" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A239" t="s">
         <v>152</v>
       </c>
@@ -8350,7 +8325,7 @@
         <v>604</v>
       </c>
     </row>
-    <row r="240" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="240" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A240" t="s">
         <v>180</v>
       </c>
@@ -8364,7 +8339,7 @@
         <v>602</v>
       </c>
     </row>
-    <row r="241" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="241" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A241" t="s">
         <v>308</v>
       </c>
@@ -8378,7 +8353,7 @@
         <v>604</v>
       </c>
     </row>
-    <row r="242" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="242" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A242" t="s">
         <v>215</v>
       </c>
@@ -8391,11 +8366,8 @@
       <c r="D242" t="s">
         <v>606</v>
       </c>
-      <c r="E242" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="243" spans="1:5" x14ac:dyDescent="0.25">
+    </row>
+    <row r="243" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A243" t="s">
         <v>43</v>
       </c>
@@ -8409,7 +8381,7 @@
         <v>600</v>
       </c>
     </row>
-    <row r="244" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="244" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A244" t="s">
         <v>64</v>
       </c>
@@ -8423,7 +8395,7 @@
         <v>600</v>
       </c>
     </row>
-    <row r="245" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="245" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A245" t="s">
         <v>405</v>
       </c>
@@ -8437,7 +8409,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="246" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="246" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A246" t="s">
         <v>62</v>
       </c>
@@ -8451,7 +8423,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="247" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="247" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A247" t="s">
         <v>297</v>
       </c>
@@ -8465,7 +8437,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="248" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="248" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A248" t="s">
         <v>98</v>
       </c>
@@ -8479,7 +8451,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="249" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="249" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A249" t="s">
         <v>120</v>
       </c>
@@ -8493,7 +8465,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="250" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="250" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A250" t="s">
         <v>15</v>
       </c>
@@ -8507,7 +8479,7 @@
         <v>604</v>
       </c>
     </row>
-    <row r="251" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="251" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A251" t="s">
         <v>18</v>
       </c>
@@ -8520,11 +8492,8 @@
       <c r="D251" t="s">
         <v>606</v>
       </c>
-      <c r="E251" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="252" spans="1:5" x14ac:dyDescent="0.25">
+    </row>
+    <row r="252" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A252" t="s">
         <v>48</v>
       </c>
@@ -8538,7 +8507,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="253" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="253" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A253" t="s">
         <v>268</v>
       </c>
@@ -8552,7 +8521,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="254" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="254" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A254" t="s">
         <v>109</v>
       </c>
@@ -8566,7 +8535,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="255" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="255" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A255" t="s">
         <v>23</v>
       </c>
@@ -8580,7 +8549,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="256" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="256" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A256" t="s">
         <v>32</v>
       </c>
@@ -8593,11 +8562,8 @@
       <c r="D256" t="s">
         <v>606</v>
       </c>
-      <c r="E256" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="257" spans="1:5" x14ac:dyDescent="0.25">
+    </row>
+    <row r="257" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A257" t="s">
         <v>59</v>
       </c>
@@ -8611,7 +8577,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="258" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="258" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A258" t="s">
         <v>34</v>
       </c>
@@ -8625,7 +8591,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="259" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="259" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A259" t="s">
         <v>84</v>
       </c>
@@ -8639,7 +8605,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="260" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="260" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A260" t="s">
         <v>293</v>
       </c>
@@ -8653,7 +8619,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="261" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="261" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A261" t="s">
         <v>294</v>
       </c>
@@ -8667,7 +8633,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="262" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="262" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A262" t="s">
         <v>335</v>
       </c>
@@ -8681,7 +8647,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="263" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="263" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A263" t="s">
         <v>311</v>
       </c>
@@ -8695,7 +8661,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="264" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="264" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A264" t="s">
         <v>292</v>
       </c>
@@ -8709,7 +8675,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="265" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="265" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A265" t="s">
         <v>128</v>
       </c>
@@ -8723,7 +8689,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="266" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="266" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A266" t="s">
         <v>60</v>
       </c>
@@ -8736,11 +8702,8 @@
       <c r="D266" t="s">
         <v>606</v>
       </c>
-      <c r="E266" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="267" spans="1:5" x14ac:dyDescent="0.25">
+    </row>
+    <row r="267" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A267" t="s">
         <v>150</v>
       </c>
@@ -8754,7 +8717,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="268" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="268" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A268" t="s">
         <v>131</v>
       </c>
@@ -8768,7 +8731,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="269" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="269" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A269" t="s">
         <v>244</v>
       </c>
@@ -8782,7 +8745,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="270" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="270" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A270" t="s">
         <v>44</v>
       </c>
@@ -8796,7 +8759,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="271" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="271" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A271" t="s">
         <v>40</v>
       </c>
@@ -8810,7 +8773,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="272" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="272" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A272" t="s">
         <v>204</v>
       </c>
@@ -9720,7 +9683,7 @@
         <v>600</v>
       </c>
     </row>
-    <row r="337" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="337" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A337" t="s">
         <v>301</v>
       </c>
@@ -9734,7 +9697,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="338" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="338" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A338" t="s">
         <v>258</v>
       </c>
@@ -9748,7 +9711,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="339" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="339" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A339" t="s">
         <v>404</v>
       </c>
@@ -9762,7 +9725,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="340" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="340" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A340" t="s">
         <v>78</v>
       </c>
@@ -9776,7 +9739,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="341" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="341" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A341" t="s">
         <v>0</v>
       </c>
@@ -9789,11 +9752,8 @@
       <c r="D341" t="s">
         <v>606</v>
       </c>
-      <c r="E341" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="342" spans="1:5" x14ac:dyDescent="0.25">
+    </row>
+    <row r="342" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A342" t="s">
         <v>299</v>
       </c>
@@ -9807,7 +9767,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="343" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="343" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A343" t="s">
         <v>25</v>
       </c>
@@ -9821,7 +9781,7 @@
         <v>600</v>
       </c>
     </row>
-    <row r="344" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="344" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A344" t="s">
         <v>46</v>
       </c>
@@ -9834,11 +9794,8 @@
       <c r="D344" t="s">
         <v>606</v>
       </c>
-      <c r="E344" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="345" spans="1:5" x14ac:dyDescent="0.25">
+    </row>
+    <row r="345" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A345" t="s">
         <v>75</v>
       </c>
@@ -9852,7 +9809,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="346" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="346" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A346" t="s">
         <v>82</v>
       </c>
@@ -9866,7 +9823,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="347" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="347" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A347" t="s">
         <v>68</v>
       </c>
@@ -9880,7 +9837,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="348" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="348" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A348" t="s">
         <v>135</v>
       </c>
@@ -9891,10 +9848,10 @@
         <v>582</v>
       </c>
       <c r="D348" t="s">
-        <v>606</v>
-      </c>
-    </row>
-    <row r="349" spans="1:5" x14ac:dyDescent="0.25">
+        <v>604</v>
+      </c>
+    </row>
+    <row r="349" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A349" t="s">
         <v>260</v>
       </c>
@@ -9908,7 +9865,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="350" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="350" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A350" t="s">
         <v>153</v>
       </c>
@@ -9921,11 +9878,8 @@
       <c r="D350" t="s">
         <v>606</v>
       </c>
-      <c r="E350" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="351" spans="1:5" x14ac:dyDescent="0.25">
+    </row>
+    <row r="351" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A351" t="s">
         <v>226</v>
       </c>
@@ -9939,7 +9893,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="352" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="352" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A352" t="s">
         <v>296</v>
       </c>
@@ -10889,6 +10843,104 @@
       </c>
       <c r="D419" t="s">
         <v>604</v>
+      </c>
+    </row>
+    <row r="420" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A420" t="s">
+        <v>610</v>
+      </c>
+      <c r="B420" t="s">
+        <v>428</v>
+      </c>
+      <c r="C420" t="s">
+        <v>582</v>
+      </c>
+      <c r="D420" t="s">
+        <v>602</v>
+      </c>
+    </row>
+    <row r="421" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A421" t="s">
+        <v>611</v>
+      </c>
+      <c r="B421" t="s">
+        <v>428</v>
+      </c>
+      <c r="C421" t="s">
+        <v>582</v>
+      </c>
+      <c r="D421" t="s">
+        <v>602</v>
+      </c>
+    </row>
+    <row r="422" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A422" t="s">
+        <v>612</v>
+      </c>
+      <c r="B422" t="s">
+        <v>428</v>
+      </c>
+      <c r="C422" t="s">
+        <v>582</v>
+      </c>
+      <c r="D422" t="s">
+        <v>602</v>
+      </c>
+    </row>
+    <row r="423" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A423" t="s">
+        <v>613</v>
+      </c>
+      <c r="B423" t="s">
+        <v>428</v>
+      </c>
+      <c r="C423" t="s">
+        <v>582</v>
+      </c>
+      <c r="D423" t="s">
+        <v>602</v>
+      </c>
+    </row>
+    <row r="424" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A424" t="s">
+        <v>614</v>
+      </c>
+      <c r="B424" t="s">
+        <v>428</v>
+      </c>
+      <c r="C424" t="s">
+        <v>582</v>
+      </c>
+      <c r="D424" t="s">
+        <v>602</v>
+      </c>
+    </row>
+    <row r="425" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A425" t="s">
+        <v>615</v>
+      </c>
+      <c r="B425" t="s">
+        <v>428</v>
+      </c>
+      <c r="C425" t="s">
+        <v>582</v>
+      </c>
+      <c r="D425" t="s">
+        <v>602</v>
+      </c>
+    </row>
+    <row r="426" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A426" t="s">
+        <v>616</v>
+      </c>
+      <c r="B426" t="s">
+        <v>428</v>
+      </c>
+      <c r="C426" t="s">
+        <v>582</v>
+      </c>
+      <c r="D426" t="s">
+        <v>602</v>
       </c>
     </row>
   </sheetData>

</xml_diff>